<commit_message>
HE missing acc part 2
</commit_message>
<xml_diff>
--- a/data/hex_xlsx/KNEBV.HE.xlsx
+++ b/data/hex_xlsx/KNEBV.HE.xlsx
@@ -13660,13 +13660,25 @@
       <c r="Q68" s="20">
         <v>1595.73</v>
       </c>
-      <c r="R68" s="15"/>
-      <c r="S68" s="15"/>
-      <c r="T68" s="15"/>
+      <c r="R68" s="20">
+        <f t="shared" ref="R68:T68" si="1">R69+R72+R76+R83+R91</f>
+        <v>1659.59</v>
+      </c>
+      <c r="S68" s="20">
+        <f t="shared" si="1"/>
+        <v>2079.48</v>
+      </c>
+      <c r="T68" s="20">
+        <f t="shared" si="1"/>
+        <v>1587.31</v>
+      </c>
       <c r="U68" s="20">
         <v>1790.53</v>
       </c>
-      <c r="V68" s="15"/>
+      <c r="V68" s="20">
+        <f>V69+V72+V76+V83+V91</f>
+        <v>1711.85</v>
+      </c>
       <c r="W68" s="20">
         <v>1538.83</v>
       </c>

</xml_diff>